<commit_message>
Redesign fighter onboarding and rankings with private gym connections
</commit_message>
<xml_diff>
--- a/docs/templates/RFC-rankings-template.xlsx
+++ b/docs/templates/RFC-rankings-template.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rankings'!$A$1:$D$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fighters'!$A$1:$D$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rankings'!$A$1:$D$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fighters'!$A$1:$D$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00123C2B"/>
+        <fgColor rgb="00181818"/>
       </patternFill>
     </fill>
   </fills>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -765,134 +765,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>20</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Diego Santos</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>21</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Harvey Blake</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>22</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Niall Doyle</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Marco Costa</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>23</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Enzo Ricci</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Daniel Cole</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Caleb Moore</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D25"/>
+  <autoFilter ref="A1:D18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -903,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1240,134 +1114,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>24</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Caleb Moore</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>3</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Daniel Cole</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Diego Santos</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>23</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Enzo Ricci</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Harvey Blake</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Marco Costa</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Niall Doyle</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Welterweight</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D25"/>
+  <autoFilter ref="A1:D18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1378,7 +1126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -1394,68 +1142,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Edit the Rankings sheet only. Keep athlete_id, name, division, position headers.</t>
+          <t>Active categories: Featherweight and Lightweight only.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Use existing athlete IDs from the Fighters reference sheet. Name and division must match that athlete.</t>
+          <t>Edit the Rankings sheet only. Keep athlete_id, name, division, position headers.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Each represented division replaces that entire division ranking. Omitted divisions stay unchanged.</t>
+          <t>Use existing athlete IDs from the Fighters reference sheet. Name and division must match that athlete.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Within each division: one athlete per row; unique positions 1, 2, 3 … without gaps.</t>
+          <t>Each represented division replaces that entire division ranking. Omitted divisions stay unchanged.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>To add a currently unranked athlete, add its ID, exact name, division and desired position.</t>
+          <t>Within each division: one athlete per row; unique positions 1, 2, 3 … without gaps.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Do not use formulas, macros, duplicate fighters, blank required cells or invented athlete IDs.</t>
+          <t>To add a currently unranked athlete, add its ID, exact name, division and desired position.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Save as .xlsx. Maximum file size 512 KiB; maximum 2,000 ranking rows.</t>
+          <t>Do not use formulas, macros, duplicate fighters, blank required cells or invented athlete IDs.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Upload as app admin, review the preview and removals, then explicitly confirm publication.</t>
+          <t>Save as .xlsx. Maximum file size 512 KiB; maximum 2,000 ranking rows.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>An empty file cannot erase rankings. Unlisted athletes in a represented division become unranked.</t>
+          <t>Upload as app admin, review the preview and removals, then explicitly confirm publication.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>An empty file cannot erase rankings. Unlisted athletes in a represented division become unranked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>This upload changes rankings only; it does not change fight records or create athletes.</t>
         </is>

</xml_diff>